<commit_message>
2026 06 16 update
</commit_message>
<xml_diff>
--- a/httpdocs/template/henko_temp.xlsx
+++ b/httpdocs/template/henko_temp.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\kotei3\httpdocs\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\hochiki\httpdocs\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078B6E34-3F19-4E33-9FBB-084DC8B90D46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1710" yWindow="1155" windowWidth="15600" windowHeight="12705"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>202●年 ●月 吉日</t>
   </si>
@@ -52,12 +53,15 @@
   </si>
   <si>
     <t>●●マンション 作業工程表</t>
+  </si>
+  <si>
+    <t>ステータス</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="15">
     <font>
       <sz val="11"/>
@@ -238,25 +242,25 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="標準 3" xfId="1"/>
+    <cellStyle name="標準 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
@@ -272,9 +276,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -312,9 +316,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -349,7 +353,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -384,7 +388,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -557,71 +561,72 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BB10"/>
-  <sheetFormatPr defaultColWidth="7.5" defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultColWidth="7.5" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="0.75" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7.75" style="1" customWidth="1"/>
+    <col min="1" max="1" width="0.69921875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.3984375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="7.69921875" style="1" customWidth="1"/>
     <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.25" style="2" customWidth="1"/>
-    <col min="8" max="8" width="13.125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.09765625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.3984375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.19921875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="13.09765625" style="2" customWidth="1"/>
     <col min="9" max="9" width="10.5" style="2" customWidth="1"/>
-    <col min="10" max="10" width="11.75" style="2" customWidth="1"/>
-    <col min="11" max="18" width="5.125" style="2" customWidth="1"/>
-    <col min="19" max="19" width="5.125" style="3" customWidth="1"/>
-    <col min="20" max="28" width="5.125" style="2" customWidth="1"/>
-    <col min="29" max="41" width="5.125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="11.69921875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="11.5" style="2" customWidth="1"/>
+    <col min="12" max="18" width="5.09765625" style="2" customWidth="1"/>
+    <col min="19" max="19" width="5.09765625" style="3" customWidth="1"/>
+    <col min="20" max="28" width="5.09765625" style="2" customWidth="1"/>
+    <col min="29" max="41" width="5.09765625" style="1" customWidth="1"/>
     <col min="42" max="16384" width="7.5" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:54">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
     </row>
     <row r="2" spans="1:54">
       <c r="B2" s="4"/>
     </row>
-    <row r="3" spans="1:54" s="8" customFormat="1" ht="40.9" customHeight="1">
-      <c r="A3" s="22" t="s">
+    <row r="3" spans="1:54" s="8" customFormat="1" ht="40.950000000000003" customHeight="1">
+      <c r="A3" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="25"/>
-      <c r="N3" s="25"/>
-      <c r="O3" s="25"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="25"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
       <c r="R3" s="5"/>
       <c r="S3" s="3"/>
       <c r="T3" s="5"/>
@@ -710,34 +715,36 @@
       <c r="BB4" s="7"/>
     </row>
     <row r="5" spans="1:54" s="10" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="G5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="I5" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="23" t="s">
+      <c r="J5" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="7"/>
+      <c r="K5" s="21" t="s">
+        <v>11</v>
+      </c>
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
@@ -949,6 +956,6 @@
   </mergeCells>
   <phoneticPr fontId="7"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" copies="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>